<commit_message>
coal flex pilot and 216 TS
</commit_message>
<xml_diff>
--- a/VerveStacks_ZAF_grids_kan/SysSettings.xlsx
+++ b/VerveStacks_ZAF_grids_kan/SysSettings.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\VerveStacks_ZAF_grids_kan\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_ZAF_grids_kan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C891262C-C5FE-4426-98DB-F84B8931DAEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6394675F-86A8-43AA-A141-0CB868272980}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2452" uniqueCount="737">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2451" uniqueCount="736">
   <si>
     <t>~BookRegions_Map</t>
   </si>
@@ -2199,9 +2199,6 @@
   </si>
   <si>
     <t>H10</t>
-  </si>
-  <si>
-    <t>DeActivated</t>
   </si>
   <si>
     <t>S01,S02,S03,S04,S05,S06,S07,S08,S09,S10,S11,S12</t>
@@ -4614,11 +4611,8 @@
       <c r="B2" t="s">
         <v>0</v>
       </c>
-      <c r="F2" t="s">
+      <c r="M2" t="s">
         <v>3</v>
-      </c>
-      <c r="M2" t="s">
-        <v>720</v>
       </c>
     </row>
     <row r="3" spans="2:17">
@@ -4691,7 +4685,7 @@
         <v>705</v>
       </c>
       <c r="P4" t="s">
-        <v>721</v>
+        <v>720</v>
       </c>
       <c r="Q4" t="s">
         <v>704</v>
@@ -4771,7 +4765,7 @@
         <v>713</v>
       </c>
       <c r="O8" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="Q8" t="s">
         <v>704</v>
@@ -4805,7 +4799,7 @@
         <v>704</v>
       </c>
       <c r="M10" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="O10" t="s">
         <v>716</v>
@@ -4822,7 +4816,7 @@
         <v>704</v>
       </c>
       <c r="M11" t="s">
-        <v>724</v>
+        <v>723</v>
       </c>
       <c r="O11" t="s">
         <v>717</v>
@@ -4839,7 +4833,7 @@
         <v>704</v>
       </c>
       <c r="M12" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="O12" t="s">
         <v>718</v>
@@ -4850,7 +4844,7 @@
     </row>
     <row r="13" spans="2:17">
       <c r="M13" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
       <c r="O13" t="s">
         <v>719</v>
@@ -4861,10 +4855,10 @@
     </row>
     <row r="14" spans="2:17">
       <c r="M14" t="s">
+        <v>726</v>
+      </c>
+      <c r="O14" t="s">
         <v>727</v>
-      </c>
-      <c r="O14" t="s">
-        <v>728</v>
       </c>
       <c r="Q14" t="s">
         <v>704</v>
@@ -4872,10 +4866,10 @@
     </row>
     <row r="15" spans="2:17">
       <c r="M15" t="s">
+        <v>728</v>
+      </c>
+      <c r="O15" t="s">
         <v>729</v>
-      </c>
-      <c r="O15" t="s">
-        <v>730</v>
       </c>
       <c r="Q15" t="s">
         <v>704</v>
@@ -4883,7 +4877,7 @@
     </row>
     <row r="16" spans="2:17">
       <c r="O16" t="s">
-        <v>731</v>
+        <v>730</v>
       </c>
       <c r="Q16" t="s">
         <v>704</v>
@@ -4891,7 +4885,7 @@
     </row>
     <row r="17" spans="15:17">
       <c r="O17" t="s">
-        <v>732</v>
+        <v>731</v>
       </c>
       <c r="Q17" t="s">
         <v>704</v>
@@ -4899,7 +4893,7 @@
     </row>
     <row r="18" spans="15:17">
       <c r="O18" t="s">
-        <v>733</v>
+        <v>732</v>
       </c>
       <c r="Q18" t="s">
         <v>704</v>
@@ -4907,7 +4901,7 @@
     </row>
     <row r="19" spans="15:17">
       <c r="O19" t="s">
-        <v>734</v>
+        <v>733</v>
       </c>
       <c r="Q19" t="s">
         <v>704</v>
@@ -4915,7 +4909,7 @@
     </row>
     <row r="20" spans="15:17">
       <c r="O20" t="s">
-        <v>735</v>
+        <v>734</v>
       </c>
       <c r="Q20" t="s">
         <v>704</v>
@@ -4923,7 +4917,7 @@
     </row>
     <row r="21" spans="15:17">
       <c r="O21" t="s">
-        <v>736</v>
+        <v>735</v>
       </c>
       <c r="Q21" t="s">
         <v>704</v>

</xml_diff>